<commit_message>
feat(mapa): abreviação e cores dinâmicas via CONFIG + melhorias na tabela resumo
- reader.js: lê coluna C do CONFIG como abreviação customizada por categoria
- mapa.js: getCatAbrev consulta DB.categorias antes do fallback hardcoded
- mapa.js: buildLegenda usa c.cor diretamente (evita mismatch de nome)
- mapa.js: buildLegenda exportada para reutilização no PDF
- mapa.js: buildResumoGeral com bordas, dot colorido, zebrado e colunas compactas
- pages.js: legenda do PDF substituída por buildLegenda() dinâmica
- templates: atualização dos arquivos BASE_SEMANAL com coluna de abreviação no CONFIG

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/BASE_SEMANAL_DADOS.xlsx
+++ b/templates/BASE_SEMANAL_DADOS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://trinuscapital-my.sharepoint.com/personal/mateus_monteiro_trinusco_com_br/Documents/Área de Trabalho/TEMPORARIO/SEMANAL - ENTREGA/Relatorios/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="69" documentId="11_C7687B5054A33544D9B01B6F03B42F07F57BE01D" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AAD0218F-49AE-4DBF-B3D1-3F75F5289E19}"/>
+  <xr:revisionPtr revIDLastSave="122" documentId="11_C7687B5054A33544D9B01B6F03B42F07F57BE01D" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{002C6BB2-7FBF-4380-B4E1-D380137729AF}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1168" uniqueCount="345">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1180" uniqueCount="357">
   <si>
     <t>CHECKLIST DE ÁREA COMUM</t>
   </si>
@@ -1077,6 +1077,42 @@
   </si>
   <si>
     <t>Trinus Co.</t>
+  </si>
+  <si>
+    <t>COR</t>
+  </si>
+  <si>
+    <t>#217A3C</t>
+  </si>
+  <si>
+    <t>#1A6EE8</t>
+  </si>
+  <si>
+    <t>#E2E8F0</t>
+  </si>
+  <si>
+    <t>#800000</t>
+  </si>
+  <si>
+    <t>#FFCC66</t>
+  </si>
+  <si>
+    <t>ABREV</t>
+  </si>
+  <si>
+    <t>REST.</t>
+  </si>
+  <si>
+    <t>REPROV.</t>
+  </si>
+  <si>
+    <t>APROV</t>
+  </si>
+  <si>
+    <t>LIB</t>
+  </si>
+  <si>
+    <t>EST</t>
   </si>
 </sst>
 </file>
@@ -1088,7 +1124,7 @@
     <numFmt numFmtId="164" formatCode="0&quot;%&quot;"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="13" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1164,8 +1200,20 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="9">
+  <fills count="14">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1205,6 +1253,36 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="3" tint="0.89999084444715716"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF217A3C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1A6EE8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE2E8F0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF800000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC66"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1344,7 +1422,7 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -1410,6 +1488,24 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="165" fontId="1" fillId="8" borderId="0" xfId="2" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="11" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -1763,6 +1859,18 @@
       <tableStyleElement type="firstColumnStripe" dxfId="36"/>
     </tableStyle>
   </tableStyles>
+  <colors>
+    <mruColors>
+      <color rgb="FFFFCC66"/>
+      <color rgb="FF800000"/>
+      <color rgb="FFDC2626"/>
+      <color rgb="FFB91C1C"/>
+      <color rgb="FFEBF3FB"/>
+      <color rgb="FFE2E8F0"/>
+      <color rgb="FF1A6EE8"/>
+      <color rgb="FF217A3C"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -2208,60 +2316,108 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:A11"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="56.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B1" s="10"/>
+      <c r="C1" s="10"/>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="20" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="3" spans="1:1" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2" s="20"/>
+      <c r="C2" s="20"/>
+    </row>
+    <row r="3" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B3" s="9" t="s">
+        <v>345</v>
+      </c>
+      <c r="C3" s="9" t="s">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B4" s="27" t="s">
+        <v>346</v>
+      </c>
+      <c r="C4" s="8" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="8" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B5" s="28" t="s">
+        <v>347</v>
+      </c>
+      <c r="C5" s="8" t="s">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="8" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B6" s="30" t="s">
+        <v>348</v>
+      </c>
+      <c r="C6" s="8" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="8" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B7" s="32" t="s">
+        <v>350</v>
+      </c>
+      <c r="C7" s="8" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="8" t="s">
         <v>102</v>
       </c>
-    </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B8" s="31" t="s">
+        <v>349</v>
+      </c>
+      <c r="C8" s="8" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="8"/>
-    </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B9" s="29"/>
+      <c r="C9" s="8"/>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="8"/>
-    </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B10" s="29"/>
+      <c r="C10" s="8"/>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="8"/>
+      <c r="B11" s="29"/>
+      <c r="C11" s="8"/>
     </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
@@ -2278,16 +2434,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="29" t="s">
+      <c r="A1" s="35" t="s">
         <v>47</v>
       </c>
-      <c r="B1" s="28"/>
+      <c r="B1" s="34"/>
     </row>
     <row r="2" spans="1:2" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="27" t="s">
+      <c r="A2" s="33" t="s">
         <v>48</v>
       </c>
-      <c r="B2" s="28"/>
+      <c r="B2" s="34"/>
     </row>
     <row r="3" spans="1:2" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
@@ -2322,10 +2478,10 @@
       </c>
     </row>
     <row r="7" spans="1:2" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="27" t="s">
+      <c r="A7" s="33" t="s">
         <v>56</v>
       </c>
-      <c r="B7" s="28"/>
+      <c r="B7" s="34"/>
     </row>
     <row r="8" spans="1:2" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
@@ -2354,10 +2510,10 @@
       </c>
     </row>
     <row r="11" spans="1:2" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="27" t="s">
+      <c r="A11" s="33" t="s">
         <v>60</v>
       </c>
-      <c r="B11" s="28"/>
+      <c r="B11" s="34"/>
     </row>
     <row r="12" spans="1:2" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
@@ -2365,7 +2521,7 @@
       </c>
       <c r="B12" s="6">
         <f>COUNTIF(Tabela2[CATEGORIA],"Aprovou Vistoria")</f>
-        <v>42</v>
+        <v>39</v>
       </c>
     </row>
     <row r="13" spans="1:2" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -2383,7 +2539,7 @@
       </c>
       <c r="B14" s="7">
         <f>IF(B13=0,"",ROUND(B12/B13*100,0))</f>
-        <v>53</v>
+        <v>49</v>
       </c>
     </row>
   </sheetData>
@@ -2409,12 +2565,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="30" t="s">
+      <c r="A1" s="36" t="s">
         <v>64</v>
       </c>
-      <c r="B1" s="28"/>
-      <c r="C1" s="28"/>
-      <c r="D1" s="28"/>
+      <c r="B1" s="34"/>
+      <c r="C1" s="34"/>
+      <c r="D1" s="34"/>
     </row>
     <row r="2" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="21" t="s">
@@ -2707,7 +2863,7 @@
         <v>163</v>
       </c>
       <c r="D22" t="s">
-        <v>45</v>
+        <v>102</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
@@ -2721,7 +2877,7 @@
         <v>164</v>
       </c>
       <c r="D23" t="s">
-        <v>43</v>
+        <v>102</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
@@ -2735,7 +2891,7 @@
         <v>161</v>
       </c>
       <c r="D24" t="s">
-        <v>44</v>
+        <v>102</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
@@ -2749,7 +2905,7 @@
         <v>162</v>
       </c>
       <c r="D25" t="s">
-        <v>43</v>
+        <v>102</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
@@ -2763,7 +2919,7 @@
         <v>163</v>
       </c>
       <c r="D26" t="s">
-        <v>43</v>
+        <v>102</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
@@ -2777,7 +2933,7 @@
         <v>164</v>
       </c>
       <c r="D27" t="s">
-        <v>45</v>
+        <v>102</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
@@ -3602,14 +3758,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="30" t="s">
+      <c r="A1" s="36" t="s">
         <v>92</v>
       </c>
-      <c r="B1" s="28"/>
-      <c r="C1" s="28"/>
-      <c r="D1" s="28"/>
-      <c r="E1" s="28"/>
-      <c r="F1" s="28"/>
+      <c r="B1" s="34"/>
+      <c r="C1" s="34"/>
+      <c r="D1" s="34"/>
+      <c r="E1" s="34"/>
+      <c r="F1" s="34"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="15" t="s">
@@ -9459,17 +9615,17 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="30" t="s">
+      <c r="A1" s="36" t="s">
         <v>107</v>
       </c>
-      <c r="B1" s="30"/>
-      <c r="C1" s="30"/>
-      <c r="D1" s="30"/>
-      <c r="E1" s="30"/>
-      <c r="F1" s="30"/>
-      <c r="G1" s="30"/>
-      <c r="H1" s="30"/>
-      <c r="I1" s="30"/>
+      <c r="B1" s="36"/>
+      <c r="C1" s="36"/>
+      <c r="D1" s="36"/>
+      <c r="E1" s="36"/>
+      <c r="F1" s="36"/>
+      <c r="G1" s="36"/>
+      <c r="H1" s="36"/>
+      <c r="I1" s="36"/>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="21" t="s">
@@ -9844,42 +10000,42 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="30" t="s">
+      <c r="A1" s="36" t="s">
         <v>107</v>
       </c>
-      <c r="B1" s="28"/>
-      <c r="C1" s="28"/>
-      <c r="D1" s="28"/>
-      <c r="E1" s="28"/>
-      <c r="F1" s="28"/>
-      <c r="G1" s="28"/>
-      <c r="H1" s="28"/>
-      <c r="I1" s="28"/>
-      <c r="J1" s="28"/>
-      <c r="K1" s="28"/>
-      <c r="L1" s="28"/>
-      <c r="M1" s="28"/>
-      <c r="N1" s="28"/>
-      <c r="O1" s="28"/>
+      <c r="B1" s="34"/>
+      <c r="C1" s="34"/>
+      <c r="D1" s="34"/>
+      <c r="E1" s="34"/>
+      <c r="F1" s="34"/>
+      <c r="G1" s="34"/>
+      <c r="H1" s="34"/>
+      <c r="I1" s="34"/>
+      <c r="J1" s="34"/>
+      <c r="K1" s="34"/>
+      <c r="L1" s="34"/>
+      <c r="M1" s="34"/>
+      <c r="N1" s="34"/>
+      <c r="O1" s="34"/>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A2" s="31" t="s">
+      <c r="A2" s="37" t="s">
         <v>140</v>
       </c>
-      <c r="B2" s="32"/>
-      <c r="C2" s="32"/>
-      <c r="D2" s="32"/>
-      <c r="E2" s="32"/>
-      <c r="F2" s="32"/>
-      <c r="G2" s="32"/>
-      <c r="H2" s="32"/>
-      <c r="I2" s="32"/>
-      <c r="J2" s="32"/>
-      <c r="K2" s="32"/>
-      <c r="L2" s="32"/>
-      <c r="M2" s="32"/>
-      <c r="N2" s="32"/>
-      <c r="O2" s="33"/>
+      <c r="B2" s="38"/>
+      <c r="C2" s="38"/>
+      <c r="D2" s="38"/>
+      <c r="E2" s="38"/>
+      <c r="F2" s="38"/>
+      <c r="G2" s="38"/>
+      <c r="H2" s="38"/>
+      <c r="I2" s="38"/>
+      <c r="J2" s="38"/>
+      <c r="K2" s="38"/>
+      <c r="L2" s="38"/>
+      <c r="M2" s="38"/>
+      <c r="N2" s="38"/>
+      <c r="O2" s="39"/>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3" s="11" t="s">
@@ -11410,130 +11566,130 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="30" t="s">
+      <c r="A1" s="36" t="s">
         <v>155</v>
       </c>
-      <c r="B1" s="28"/>
-      <c r="C1" s="28"/>
-      <c r="D1" s="28"/>
+      <c r="B1" s="34"/>
+      <c r="C1" s="34"/>
+      <c r="D1" s="34"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="34" t="s">
+      <c r="A2" s="40" t="s">
         <v>156</v>
       </c>
-      <c r="B2" s="35"/>
-      <c r="C2" s="35"/>
-      <c r="D2" s="36"/>
+      <c r="B2" s="41"/>
+      <c r="C2" s="41"/>
+      <c r="D2" s="42"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="37" t="s">
+      <c r="A3" s="43" t="s">
         <v>339</v>
       </c>
-      <c r="B3" s="32"/>
-      <c r="C3" s="32"/>
-      <c r="D3" s="33"/>
+      <c r="B3" s="38"/>
+      <c r="C3" s="38"/>
+      <c r="D3" s="39"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" s="38"/>
-      <c r="B4" s="28"/>
-      <c r="C4" s="28"/>
-      <c r="D4" s="39"/>
+      <c r="A4" s="44"/>
+      <c r="B4" s="34"/>
+      <c r="C4" s="34"/>
+      <c r="D4" s="45"/>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" s="38"/>
-      <c r="B5" s="28"/>
-      <c r="C5" s="28"/>
-      <c r="D5" s="39"/>
+      <c r="A5" s="44"/>
+      <c r="B5" s="34"/>
+      <c r="C5" s="34"/>
+      <c r="D5" s="45"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" s="38"/>
-      <c r="B6" s="28"/>
-      <c r="C6" s="28"/>
-      <c r="D6" s="39"/>
+      <c r="A6" s="44"/>
+      <c r="B6" s="34"/>
+      <c r="C6" s="34"/>
+      <c r="D6" s="45"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" s="38"/>
-      <c r="B7" s="28"/>
-      <c r="C7" s="28"/>
-      <c r="D7" s="39"/>
+      <c r="A7" s="44"/>
+      <c r="B7" s="34"/>
+      <c r="C7" s="34"/>
+      <c r="D7" s="45"/>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8" s="38"/>
-      <c r="B8" s="28"/>
-      <c r="C8" s="28"/>
-      <c r="D8" s="39"/>
+      <c r="A8" s="44"/>
+      <c r="B8" s="34"/>
+      <c r="C8" s="34"/>
+      <c r="D8" s="45"/>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" s="38"/>
-      <c r="B9" s="28"/>
-      <c r="C9" s="28"/>
-      <c r="D9" s="39"/>
+      <c r="A9" s="44"/>
+      <c r="B9" s="34"/>
+      <c r="C9" s="34"/>
+      <c r="D9" s="45"/>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A10" s="38"/>
-      <c r="B10" s="28"/>
-      <c r="C10" s="28"/>
-      <c r="D10" s="39"/>
+      <c r="A10" s="44"/>
+      <c r="B10" s="34"/>
+      <c r="C10" s="34"/>
+      <c r="D10" s="45"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11" s="38"/>
-      <c r="B11" s="28"/>
-      <c r="C11" s="28"/>
-      <c r="D11" s="39"/>
+      <c r="A11" s="44"/>
+      <c r="B11" s="34"/>
+      <c r="C11" s="34"/>
+      <c r="D11" s="45"/>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12" s="38"/>
-      <c r="B12" s="28"/>
-      <c r="C12" s="28"/>
-      <c r="D12" s="39"/>
+      <c r="A12" s="44"/>
+      <c r="B12" s="34"/>
+      <c r="C12" s="34"/>
+      <c r="D12" s="45"/>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A13" s="38"/>
-      <c r="B13" s="28"/>
-      <c r="C13" s="28"/>
-      <c r="D13" s="39"/>
+      <c r="A13" s="44"/>
+      <c r="B13" s="34"/>
+      <c r="C13" s="34"/>
+      <c r="D13" s="45"/>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A14" s="38"/>
-      <c r="B14" s="28"/>
-      <c r="C14" s="28"/>
-      <c r="D14" s="39"/>
+      <c r="A14" s="44"/>
+      <c r="B14" s="34"/>
+      <c r="C14" s="34"/>
+      <c r="D14" s="45"/>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A15" s="38"/>
-      <c r="B15" s="28"/>
-      <c r="C15" s="28"/>
-      <c r="D15" s="39"/>
+      <c r="A15" s="44"/>
+      <c r="B15" s="34"/>
+      <c r="C15" s="34"/>
+      <c r="D15" s="45"/>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A16" s="38"/>
-      <c r="B16" s="28"/>
-      <c r="C16" s="28"/>
-      <c r="D16" s="39"/>
+      <c r="A16" s="44"/>
+      <c r="B16" s="34"/>
+      <c r="C16" s="34"/>
+      <c r="D16" s="45"/>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A17" s="38"/>
-      <c r="B17" s="28"/>
-      <c r="C17" s="28"/>
-      <c r="D17" s="39"/>
+      <c r="A17" s="44"/>
+      <c r="B17" s="34"/>
+      <c r="C17" s="34"/>
+      <c r="D17" s="45"/>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A18" s="38"/>
-      <c r="B18" s="28"/>
-      <c r="C18" s="28"/>
-      <c r="D18" s="39"/>
+      <c r="A18" s="44"/>
+      <c r="B18" s="34"/>
+      <c r="C18" s="34"/>
+      <c r="D18" s="45"/>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A19" s="38"/>
-      <c r="B19" s="28"/>
-      <c r="C19" s="28"/>
-      <c r="D19" s="39"/>
+      <c r="A19" s="44"/>
+      <c r="B19" s="34"/>
+      <c r="C19" s="34"/>
+      <c r="D19" s="45"/>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A20" s="40"/>
-      <c r="B20" s="41"/>
-      <c r="C20" s="41"/>
-      <c r="D20" s="42"/>
+      <c r="A20" s="46"/>
+      <c r="B20" s="47"/>
+      <c r="C20" s="47"/>
+      <c r="D20" s="48"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -11562,30 +11718,30 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="30" t="s">
+      <c r="A1" s="36" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="28"/>
-      <c r="C1" s="28"/>
-      <c r="D1" s="28"/>
-      <c r="E1" s="28"/>
-      <c r="F1" s="28"/>
-      <c r="G1" s="28"/>
-      <c r="H1" s="28"/>
-      <c r="I1" s="28"/>
+      <c r="B1" s="34"/>
+      <c r="C1" s="34"/>
+      <c r="D1" s="34"/>
+      <c r="E1" s="34"/>
+      <c r="F1" s="34"/>
+      <c r="G1" s="34"/>
+      <c r="H1" s="34"/>
+      <c r="I1" s="34"/>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A2" s="43" t="s">
+      <c r="A2" s="49" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="28"/>
-      <c r="C2" s="28"/>
-      <c r="D2" s="28"/>
-      <c r="E2" s="28"/>
-      <c r="F2" s="28"/>
-      <c r="G2" s="28"/>
-      <c r="H2" s="28"/>
-      <c r="I2" s="28"/>
+      <c r="B2" s="34"/>
+      <c r="C2" s="34"/>
+      <c r="D2" s="34"/>
+      <c r="E2" s="34"/>
+      <c r="F2" s="34"/>
+      <c r="G2" s="34"/>
+      <c r="H2" s="34"/>
+      <c r="I2" s="34"/>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="11" t="s">

</xml_diff>